<commit_message>
Fix ActiveIngredient–DrugProduct relationship (DHSOHG-3326) AB#170231
</commit_message>
<xml_diff>
--- a/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
+++ b/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB37E560-E5F9-49BB-BFC9-AF50932BE6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2468D2-0299-EA49-9377-3DC818CDA717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9630" yWindow="2730" windowWidth="25980" windowHeight="17190" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
+    <workbookView xWindow="-42760" yWindow="940" windowWidth="25980" windowHeight="17200" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Strength</t>
-  </si>
-  <si>
     <t>Form</t>
   </si>
   <si>
@@ -70,9 +67,6 @@
     <t>{d.records[i].practitioner}</t>
   </si>
   <si>
-    <t>{d.records[i].strength}</t>
-  </si>
-  <si>
     <t>{d.records[i].form}</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
   </si>
   <si>
     <t>{d.records[i+1].quantity}</t>
-  </si>
-  <si>
-    <t>{d.records[i+1].strength}</t>
   </si>
   <si>
     <t>{d.records[i+1].form}</t>
@@ -185,9 +176,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -225,7 +216,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -331,7 +322,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -473,7 +464,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -481,17 +472,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60882D5E-E61D-5940-8D5B-09478E4A9588}">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.25" customWidth="1"/>
-    <col min="3" max="5" width="35.75" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="30.75" customWidth="1"/>
-    <col min="9" max="9" width="44.25" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="3" max="5" width="35.6640625" customWidth="1"/>
+    <col min="7" max="7" width="30.6640625" customWidth="1"/>
+    <col min="8" max="8" width="44.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -516,66 +506,57 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>18</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Active Ingredients table to Medication timeline entry card (DHSOHG-3326) for AB#17031 (#6631)
* Fix ActiveIngredient–DrugProduct relationship (DHSOHG-3326) AB#170231

* Add defensive checks for large PDF report downloads for AB#17031

* Add controller and service for drug lookup by DIN for AB#17031

* Add Active Ingredients table to Medication Entry (DHSOHG-3326) AB#17031

* Handle null CDOGS report payload for AB#170231

* Remove unused ActiveIngredient fields & improve report source AB#17031
</commit_message>
<xml_diff>
--- a/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
+++ b/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB37E560-E5F9-49BB-BFC9-AF50932BE6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2468D2-0299-EA49-9377-3DC818CDA717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9630" yWindow="2730" windowWidth="25980" windowHeight="17190" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
+    <workbookView xWindow="-42760" yWindow="940" windowWidth="25980" windowHeight="17200" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Strength</t>
-  </si>
-  <si>
     <t>Form</t>
   </si>
   <si>
@@ -70,9 +67,6 @@
     <t>{d.records[i].practitioner}</t>
   </si>
   <si>
-    <t>{d.records[i].strength}</t>
-  </si>
-  <si>
     <t>{d.records[i].form}</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
   </si>
   <si>
     <t>{d.records[i+1].quantity}</t>
-  </si>
-  <si>
-    <t>{d.records[i+1].strength}</t>
   </si>
   <si>
     <t>{d.records[i+1].form}</t>
@@ -185,9 +176,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -225,7 +216,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -331,7 +322,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -473,7 +464,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -481,17 +472,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60882D5E-E61D-5940-8D5B-09478E4A9588}">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.25" customWidth="1"/>
-    <col min="3" max="5" width="35.75" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="30.75" customWidth="1"/>
-    <col min="9" max="9" width="44.25" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="3" max="5" width="35.6640625" customWidth="1"/>
+    <col min="7" max="7" width="30.6640625" customWidth="1"/>
+    <col min="8" max="8" width="44.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -516,66 +506,57 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>18</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update medication timeline entry and report (DHSOHG-3326) AB#17031
</commit_message>
<xml_diff>
--- a/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
+++ b/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2468D2-0299-EA49-9377-3DC818CDA717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB37E560-E5F9-49BB-BFC9-AF50932BE6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-42760" yWindow="940" windowWidth="25980" windowHeight="17200" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
+    <workbookView xWindow="9630" yWindow="2730" windowWidth="25980" windowHeight="17190" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Date</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Strength</t>
+  </si>
+  <si>
     <t>Form</t>
   </si>
   <si>
@@ -67,6 +70,9 @@
     <t>{d.records[i].practitioner}</t>
   </si>
   <si>
+    <t>{d.records[i].strength}</t>
+  </si>
+  <si>
     <t>{d.records[i].form}</t>
   </si>
   <si>
@@ -83,6 +89,9 @@
   </si>
   <si>
     <t>{d.records[i+1].quantity}</t>
+  </si>
+  <si>
+    <t>{d.records[i+1].strength}</t>
   </si>
   <si>
     <t>{d.records[i+1].form}</t>
@@ -176,9 +185,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -216,7 +225,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -322,7 +331,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -464,7 +473,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -472,16 +481,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60882D5E-E61D-5940-8D5B-09478E4A9588}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="3" max="5" width="35.6640625" customWidth="1"/>
-    <col min="7" max="7" width="30.6640625" customWidth="1"/>
-    <col min="8" max="8" width="44.1640625" customWidth="1"/>
+    <col min="1" max="1" width="14.25" customWidth="1"/>
+    <col min="3" max="5" width="35.75" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="30.75" customWidth="1"/>
+    <col min="9" max="9" width="44.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,57 +516,66 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
         <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update medication timeline entry and report (DHSOHG-3326) AB#17031 (#6637)
</commit_message>
<xml_diff>
--- a/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
+++ b/Apps/GatewayApi/src/Assets/Templates/MedicationReport.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2468D2-0299-EA49-9377-3DC818CDA717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB37E560-E5F9-49BB-BFC9-AF50932BE6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-42760" yWindow="940" windowWidth="25980" windowHeight="17200" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
+    <workbookView xWindow="9630" yWindow="2730" windowWidth="25980" windowHeight="17190" xr2:uid="{F605F369-0C71-414E-B75C-5C18C8076E19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Date</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Strength</t>
+  </si>
+  <si>
     <t>Form</t>
   </si>
   <si>
@@ -67,6 +70,9 @@
     <t>{d.records[i].practitioner}</t>
   </si>
   <si>
+    <t>{d.records[i].strength}</t>
+  </si>
+  <si>
     <t>{d.records[i].form}</t>
   </si>
   <si>
@@ -83,6 +89,9 @@
   </si>
   <si>
     <t>{d.records[i+1].quantity}</t>
+  </si>
+  <si>
+    <t>{d.records[i+1].strength}</t>
   </si>
   <si>
     <t>{d.records[i+1].form}</t>
@@ -176,9 +185,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -216,7 +225,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -322,7 +331,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -464,7 +473,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -472,16 +481,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60882D5E-E61D-5940-8D5B-09478E4A9588}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="3" max="5" width="35.6640625" customWidth="1"/>
-    <col min="7" max="7" width="30.6640625" customWidth="1"/>
-    <col min="8" max="8" width="44.1640625" customWidth="1"/>
+    <col min="1" max="1" width="14.25" customWidth="1"/>
+    <col min="3" max="5" width="35.75" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="30.75" customWidth="1"/>
+    <col min="9" max="9" width="44.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,57 +516,66 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
         <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>